<commit_message>
converted english words to german as per client req
</commit_message>
<xml_diff>
--- a/excel/output.xlsx
+++ b/excel/output.xlsx
@@ -16,16 +16,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13062" uniqueCount="120">
   <si>
-    <t>Engine</t>
+    <t>Motor</t>
   </si>
   <si>
-    <t>Transmission</t>
+    <t>Getriebe</t>
   </si>
   <si>
     <t>Code</t>
   </si>
   <si>
-    <t>Price</t>
+    <t>Listenpreis1</t>
   </si>
   <si>
     <t>Feature</t>
@@ -274,7 +274,7 @@
     <t>Sicherheits- und A ssistenzsysteme Referenz START Style S TART+</t>
   </si>
   <si>
-    <t>Fahrer- und B eifahrerAirbag (mit Beifahrer-Deaktivierung), vordere S eiten- und K opfAirbags vorn und hinten (cid:127) (cid:127) (cid:127)</t>
+    <t>Fahrer- und B eifahrerairbag (mit Beifahrer-Deaktivierung), vordere S eiten- und K opfairbags vorn und hinten (cid:127) (cid:127) (cid:127)</t>
   </si>
   <si>
     <t>Kopfstützen u nd D reipunkt-Sicherheitsgurte v orn und h inten (cid:127) (cid:127) (cid:127)</t>
@@ -301,7 +301,7 @@
     <t>Manuelle K limaanlage mit Pollen- und Staubfilter - (cid:127) -</t>
   </si>
   <si>
-    <t>Climatronic a utomatische Z weizonen-Air Conditioning - - (cid:127)</t>
+    <t>Climatronic a utomatische Z weizonen-Klimaanlage - - (cid:127)</t>
   </si>
   <si>
     <t>Fahrersitz höhenverstellbar ( FR: beide V ordersitze höhenverstellbar) F R-Sportsitze (cid:127) (cid:127) (cid:127)</t>
@@ -328,10 +328,10 @@
     <t>Ambientebeleuchtung im I nnenraum, i n den Türen, d er Mittelkonsole u nd im F ußraum - - (cid:127)</t>
   </si>
   <si>
-    <t>Voll-LED-Headlights mit Tagfahrlicht (cid:127) (cid:127) (cid:127)</t>
+    <t>Voll-LED-Scheinwerfer mit Tagfahrlicht (cid:127) (cid:127) (cid:127)</t>
   </si>
   <si>
-    <t>NebelHeadlights mit Kurvenlicht (auch f ür Fahrzeuge d er Serien Reference u nd S tyle, h ergestellt bis Ende August 2026) - - (cid:127)</t>
+    <t>Nebelscheinwerfer mit Kurvenlicht (auch f ür Fahrzeuge d er Serien Reference u nd S tyle, h ergestellt bis Ende August 2026) - - (cid:127)</t>
   </si>
   <si>
     <t>LED-Rückleuchten (cid:127) (cid:127) (cid:127)</t>
@@ -349,13 +349,13 @@
     <t>Beheizbare A ußenspiegel - - (cid:127)</t>
   </si>
   <si>
-    <t>Rain Sensor - - (cid:127)</t>
+    <t>Regensensor - - (cid:127)</t>
   </si>
   <si>
-    <t>Parking Assistance vorn + Rear View Camera - - (cid:127)</t>
+    <t>Einparkhilfe vorn + Rückfahrkamera - - (cid:127)</t>
   </si>
   <si>
-    <t>Central Locking mit Fernbedienung, 15-Zoll- (cid:127) (cid:127) (cid:127)</t>
+    <t>Zentralverriegelung mit Fernbedienung, 15-Zoll- (cid:127) (cid:127) (cid:127)</t>
   </si>
   <si>
     <t>Stahlfelgen mit 185/65 R 15-Reifen ( Produktion bis M ärz 2026 – 1 5-Zoll-Leichtmetallfelgen), 1 6-Zoll-Leichtmetallfelgen (cid:127) - -</t>
@@ -380,8 +380,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -397,7 +405,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -405,12 +413,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,22 +746,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed feature column bug
</commit_message>
<xml_diff>
--- a/excel/output.xlsx
+++ b/excel/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="59">
   <si>
     <t>name</t>
   </si>
@@ -49,25 +49,16 @@
     <t>S</t>
   </si>
   <si>
-    <t>1.0 TSI 1 15 Automatik 85/ 1 15 DSG 7-Gang KJG2WZ26 20 890</t>
-  </si>
-  <si>
-    <t>1.0 TSI 1 15 Automatik 85 / 1 15 DSG 7-Gang KJG5WZ26 23 200</t>
-  </si>
-  <si>
-    <t>1.5 TSI 1 50 Automatik 110 / 150 DSG 7-Gang KJG5NZ26 24 250</t>
-  </si>
-  <si>
-    <t>Sicherheits- und A ssistenzsysteme Referenz START Style S TART+</t>
-  </si>
-  <si>
-    <t>Fahrer- und B eifahrerairbag (mit Beifahrer-Deaktivierung), vordere S eiten- und K opfairbags vorn und hinten</t>
-  </si>
-  <si>
-    <t>Kopfstützen u nd D reipunkt-Sicherheitsgurte v orn und h inten</t>
-  </si>
-  <si>
-    <t>Hintere S cheibenbremsen ( für Motoren ü ber 100.000 k m) -</t>
+    <t>Fahrer- und Beifahrerairbag (mit Beifahrer-Deaktivierung), vordere Seiten- und Kopfairbags vorn und hinten</t>
+  </si>
+  <si>
+    <t>Kopfstützen und Dreipunkt-Sicherheitsgurte v orn und h inten</t>
+  </si>
+  <si>
+    <t>Elektronisches Stabilitätsprogramm (ESC), ABS, ASR, Multikollisionsbremse</t>
+  </si>
+  <si>
+    <t>Hintere Scheibenbremsen ( für Motoren ü ber 100.000 k m) -</t>
   </si>
   <si>
     <t>Elektronische Differenzialsperre - -</t>
@@ -76,46 +67,73 @@
     <t>SEAT Fahrprofil: Lenkungs-, Gaspedal- und Getriebeeinstellungen (für D SG) - -</t>
   </si>
   <si>
-    <t>FRONT ASSIST – Ü berwachung des B ereichs vor d em Fahrzeug, einschließlich C ity-Notbremsassistent mit F ußgängererkennung</t>
-  </si>
-  <si>
-    <t>Radio mit 8,25-Zoll-Farb-Touchscreen, 4 L autsprechern ( FR 6 L autsprecher), DAB+ D igitalradioempfang</t>
+    <t>Berganfahrhilfe</t>
+  </si>
+  <si>
+    <t>FRONT ASSIST – Ü berwachung des Bereichs vor d em Fahrzeug, einschließlich City-Notbremsassistent mit Fußgängererkennung</t>
+  </si>
+  <si>
+    <t>Überprüfung d er Reifendruckänderungen</t>
+  </si>
+  <si>
+    <t>Systeme zur Erkennung v on Fahrermüdigkeit und z ur Erkennung a usgewählter Verkehrszeichen</t>
+  </si>
+  <si>
+    <t>Spurhalteassistent</t>
+  </si>
+  <si>
+    <t>Geschwindigkeitsbegrenzer (Style und F Rmit Tempomat)</t>
+  </si>
+  <si>
+    <t>Radio mit 8,25-Zoll-Farb-Touchscreen, 4 Lautsprechern ( FR 6 Lautsprecher), DAB+ Digitalradioempfang</t>
   </si>
   <si>
     <t>Bluetooth-Freisprecheinrichtung, USB-Typ-C-Anschluss</t>
   </si>
   <si>
-    <t>Manuelle K limaanlage mit Pollen- und Staubfilter - -</t>
-  </si>
-  <si>
-    <t>Climatronic a utomatische Z weizonen-Klimaanlage - -</t>
-  </si>
-  <si>
-    <t>Fahrersitz höhenverstellbar ( FR: beide V ordersitze höhenverstellbar) F R-Sportsitze</t>
-  </si>
-  <si>
-    <t>Rücksitze mit ISOFIX und T op T ether, umklappbare R ücksitzlehne (bei Style und F R im V erhältnis 1 /3 - 2/3 g eteilt)</t>
+    <t>SEAT CONNECT – Sicherheit &amp; Service + Fernzugriff, Sicherheitsdienste für 1 0 Jahre + Fernzugriffsdienste f ür 1 Jahr, e Call –</t>
+  </si>
+  <si>
+    <t>Notrufsystem u nabhängig vom Mobiltelefon</t>
+  </si>
+  <si>
+    <t>Manuelle Klimaanlage mit Pollen- und Staubfilter - -</t>
+  </si>
+  <si>
+    <t>Climatronic a utomatische Zweizonen-Klimaanlage - -</t>
+  </si>
+  <si>
+    <t>Fahrersitz höhenverstellbar ( FR: beide Vordersitze höhenverstellbar) F R-Sportsitze</t>
+  </si>
+  <si>
+    <t>- -</t>
+  </si>
+  <si>
+    <t>Rücksitze mit ISOFIXund Top Tether, umklappbare R ücksitzlehne (bei Style und F Rim Verhältnis 1 /3 - 2/3 g eteilt)</t>
   </si>
   <si>
     <t>Digitales Cockpit mit 8-Zoll-Digitalinstrumententafel</t>
   </si>
   <si>
-    <t>Komfortable T ürverkleidungen im I nnenbereich -</t>
-  </si>
-  <si>
-    <t>Anthrazitfarbene D ecke -</t>
-  </si>
-  <si>
-    <t>Elektrische Fensterheber v orn und h inten, I nnenspiegel mit automatischer B lende - -</t>
-  </si>
-  <si>
-    <t>Ambientebeleuchtung im I nnenraum, i n den Türen, d er Mittelkonsole u nd im F ußraum - -</t>
+    <t>Multifunktionslenkrad, f ür Style und F R, Leder</t>
+  </si>
+  <si>
+    <t>Komfortable T ürverkleidungen im Innenbereich -</t>
+  </si>
+  <si>
+    <t>Anthrazitfarbene Decke -</t>
+  </si>
+  <si>
+    <t>Elektrische Fensterheber v orn und h inten, Innenspiegel mit automatischer Blende - -</t>
+  </si>
+  <si>
+    <t>Ambientebeleuchtung im Innenraum, i n den Türen, d er Mittelkonsole und im Fußraum - -</t>
   </si>
   <si>
     <t>Voll-LED-Scheinwerfer mit Tagfahrlicht</t>
   </si>
   <si>
-    <t>Nebelscheinwerfer mit Kurvenlicht (auch f ür Fahrzeuge d er Serien Reference u nd S tyle, h ergestellt bis Ende August 2026) - -</t>
+    <t>Nebelscheinwerfer mit Kurvenlicht (auch f ür Fahrzeuge d er Serien Reference und Style, h ergestellt bis Ende August 2026) - -</t>
   </si>
   <si>
     <t>LED-Rückleuchten</t>
@@ -127,15 +145,24 @@
     <t>Elektrische Fensterheber v orne -</t>
   </si>
   <si>
-    <t>Elektrische Fensterheber v orne u nd h inten - -</t>
-  </si>
-  <si>
-    <t>Beheizbare A ußenspiegel - -</t>
+    <t>Elektrische Fensterheber v orne und h inten - -</t>
+  </si>
+  <si>
+    <t>Elektrisch verstellbare Außenspiegel, l ackiert, f ür F Rin g länzendem Schwarz</t>
+  </si>
+  <si>
+    <t>Beheizbare Außenspiegel - -</t>
   </si>
   <si>
     <t>Regensensor - -</t>
   </si>
   <si>
+    <t>Heckscheibenwischer</t>
+  </si>
+  <si>
+    <t>Einparkhilfe hinten</t>
+  </si>
+  <si>
     <t>Einparkhilfe vorn + Rückfahrkamera - -</t>
   </si>
   <si>
@@ -148,10 +175,13 @@
     <t>mit 195/55 R 16-Reifen -</t>
   </si>
   <si>
+    <t>Nun m uss der Defekt behoben werden.</t>
+  </si>
+  <si>
+    <t>_Sicherheit</t>
+  </si>
+  <si>
     <t>_Innen</t>
-  </si>
-  <si>
-    <t>_Sicherheit</t>
   </si>
   <si>
     <t>_Räder &amp; Co</t>
@@ -529,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -572,7 +602,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -607,7 +637,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -642,7 +672,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -677,7 +707,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -712,7 +742,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -747,7 +777,7 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -782,7 +812,7 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -817,7 +847,7 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -852,7 +882,7 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -887,7 +917,7 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -922,7 +952,7 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -957,7 +987,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -992,7 +1022,7 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1027,7 +1057,7 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1062,7 +1092,7 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -1097,7 +1127,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1132,7 +1162,7 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1167,7 +1197,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1202,7 +1232,7 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1237,7 +1267,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1272,7 +1302,7 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1307,7 +1337,7 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -1342,7 +1372,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1377,7 +1407,7 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -1412,7 +1442,7 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1447,7 +1477,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -1482,7 +1512,7 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1517,7 +1547,7 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -1552,7 +1582,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -1587,7 +1617,7 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -1622,7 +1652,7 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1657,7 +1687,7 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -1692,38 +1722,388 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34">
+        <v>1</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34">
+        <v>1</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
+      <c r="A35" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
+        <v>1</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>1</v>
+      </c>
+      <c r="K35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
+      <c r="A36" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" t="s">
+        <v>58</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36">
+        <v>1</v>
+      </c>
+      <c r="I36">
+        <v>1</v>
+      </c>
+      <c r="J36">
+        <v>1</v>
+      </c>
+      <c r="K36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
+      <c r="A37" t="s">
         <v>46</v>
       </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-      <c r="D34">
-        <v>1</v>
-      </c>
-      <c r="E34">
-        <v>1</v>
-      </c>
-      <c r="F34">
-        <v>1</v>
-      </c>
-      <c r="G34">
-        <v>1</v>
-      </c>
-      <c r="H34">
-        <v>1</v>
-      </c>
-      <c r="I34">
-        <v>1</v>
-      </c>
-      <c r="J34">
-        <v>1</v>
-      </c>
-      <c r="K34">
+      <c r="B37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37">
+        <v>1</v>
+      </c>
+      <c r="G37">
+        <v>1</v>
+      </c>
+      <c r="H37">
+        <v>1</v>
+      </c>
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37">
+        <v>1</v>
+      </c>
+      <c r="K37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
+      <c r="A38" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38">
+        <v>1</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
+        <v>1</v>
+      </c>
+      <c r="I38">
+        <v>1</v>
+      </c>
+      <c r="J38">
+        <v>1</v>
+      </c>
+      <c r="K38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
+      <c r="A39" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" t="s">
+        <v>54</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39">
+        <v>1</v>
+      </c>
+      <c r="K39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
+      <c r="A40" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" t="s">
+        <v>54</v>
+      </c>
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
+        <v>1</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="J40">
+        <v>1</v>
+      </c>
+      <c r="K40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" t="s">
+        <v>55</v>
+      </c>
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41">
+        <v>1</v>
+      </c>
+      <c r="J41">
+        <v>1</v>
+      </c>
+      <c r="K41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
+      <c r="A42" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" t="s">
+        <v>56</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
+        <v>1</v>
+      </c>
+      <c r="J42">
+        <v>1</v>
+      </c>
+      <c r="K42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="A43" t="s">
+        <v>52</v>
+      </c>
+      <c r="B43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>1</v>
+      </c>
+      <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <v>1</v>
+      </c>
+      <c r="J43">
+        <v>1</v>
+      </c>
+      <c r="K43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="A44" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" t="s">
+        <v>55</v>
+      </c>
+      <c r="C44">
+        <v>1</v>
+      </c>
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <v>1</v>
+      </c>
+      <c r="H44">
+        <v>1</v>
+      </c>
+      <c r="I44">
+        <v>1</v>
+      </c>
+      <c r="J44">
+        <v>1</v>
+      </c>
+      <c r="K44">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:K34">
+  <conditionalFormatting sqref="A2:K44">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"N/A"</formula>
     </cfRule>

</xml_diff>

<commit_message>
resolved the artifacts identified
</commit_message>
<xml_diff>
--- a/excel/output.xlsx
+++ b/excel/output.xlsx
@@ -197,16 +197,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -222,7 +214,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -230,30 +222,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,37 +537,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
resolved the words detachments
</commit_message>
<xml_diff>
--- a/excel/output.xlsx
+++ b/excel/output.xlsx
@@ -52,37 +52,37 @@
     <t>Fahrer- und Beifahrerairbag (mit Beifahrer-Deaktivierung), vordere Seiten- und Kopfairbags vorn und hinten</t>
   </si>
   <si>
-    <t>Kopfstützen und Dreipunkt-Sicherheitsgurte v orn und h inten</t>
+    <t>Kopfstützen und Dreipunkt-Sicherheitsgurte vorn und hinten</t>
   </si>
   <si>
     <t>Elektronisches Stabilitätsprogramm (ESC), ABS, ASR, Multikollisionsbremse</t>
   </si>
   <si>
-    <t>Hintere Scheibenbremsen ( für Motoren ü ber 100.000 k m) -</t>
-  </si>
-  <si>
-    <t>Elektronische Differenzialsperre - -</t>
-  </si>
-  <si>
-    <t>SEAT Fahrprofil: Lenkungs-, Gaspedal- und Getriebeeinstellungen (für D SG) - -</t>
+    <t>Hintere Scheibenbremsen ( für Motoren über 100.000 km) -</t>
+  </si>
+  <si>
+    <t>Elektronische Differenzialsperre</t>
+  </si>
+  <si>
+    <t>SEAT Fahrprofil: Lenkungs-, Gaspedal- und Getriebeeinstellungen (für DSG)</t>
   </si>
   <si>
     <t>Berganfahrhilfe</t>
   </si>
   <si>
-    <t>FRONT ASSIST – Ü berwachung des Bereichs vor d em Fahrzeug, einschließlich City-Notbremsassistent mit Fußgängererkennung</t>
-  </si>
-  <si>
-    <t>Überprüfung d er Reifendruckänderungen</t>
-  </si>
-  <si>
-    <t>Systeme zur Erkennung v on Fahrermüdigkeit und z ur Erkennung a usgewählter Verkehrszeichen</t>
+    <t>FRONT ASSIST – Überwachung des Bereichs vor dem Fahrzeug, einschließlich City-Notbremsassistent mit Fußgängererkennung</t>
+  </si>
+  <si>
+    <t>Überprüfung der Reifendruckänderungen</t>
+  </si>
+  <si>
+    <t>Systeme zur Erkennung von Fahrermüdigkeit und zur Erkennung ausgewählter Verkehrszeichen</t>
   </si>
   <si>
     <t>Spurhalteassistent</t>
   </si>
   <si>
-    <t>Geschwindigkeitsbegrenzer (Style und F Rmit Tempomat)</t>
+    <t>Geschwindigkeitsbegrenzer (Style und FRmit Tempomat)</t>
   </si>
   <si>
     <t>Radio mit 8,25-Zoll-Farb-Touchscreen, 4 Lautsprechern ( FR 6 Lautsprecher), DAB+ Digitalradioempfang</t>
@@ -91,70 +91,70 @@
     <t>Bluetooth-Freisprecheinrichtung, USB-Typ-C-Anschluss</t>
   </si>
   <si>
-    <t>SEAT CONNECT – Sicherheit &amp; Service + Fernzugriff, Sicherheitsdienste für 1 0 Jahre + Fernzugriffsdienste f ür 1 Jahr, e Call –</t>
-  </si>
-  <si>
-    <t>Notrufsystem u nabhängig vom Mobiltelefon</t>
-  </si>
-  <si>
-    <t>Manuelle Klimaanlage mit Pollen- und Staubfilter - -</t>
-  </si>
-  <si>
-    <t>Climatronic a utomatische Zweizonen-Klimaanlage - -</t>
-  </si>
-  <si>
-    <t>Fahrersitz höhenverstellbar ( FR: beide Vordersitze höhenverstellbar) F R-Sportsitze</t>
+    <t>SEAT CONNECT – Sicherheit &amp; Service + Fernzugriff, Sicherheitsdienste für 10 Jahre + Fernzugriffsdienste für 1 Jahr, e Call –</t>
+  </si>
+  <si>
+    <t>Notrufsystem unabhängig vom Mobiltelefon</t>
+  </si>
+  <si>
+    <t>Manuelle Klimaanlage mit Pollen- und Staubfilter -</t>
+  </si>
+  <si>
+    <t>Climatronic automatische Zweizonen-Klimaanlage</t>
+  </si>
+  <si>
+    <t>Fahrersitz höhenverstellbar ( FR: beide Vordersitze höhenverstellbar) FR-Sportsitze</t>
   </si>
   <si>
     <t>- -</t>
   </si>
   <si>
-    <t>Rücksitze mit ISOFIXund Top Tether, umklappbare R ücksitzlehne (bei Style und F Rim Verhältnis 1 /3 - 2/3 g eteilt)</t>
+    <t>Rücksitze mit ISOFIX und Top Tether, umklappbare Rücksitzlehne (bei Style und FRim Verhältnis 1 /3 - 2/3 geteilt)</t>
   </si>
   <si>
     <t>Digitales Cockpit mit 8-Zoll-Digitalinstrumententafel</t>
   </si>
   <si>
-    <t>Multifunktionslenkrad, f ür Style und F R, Leder</t>
-  </si>
-  <si>
-    <t>Komfortable T ürverkleidungen im Innenbereich -</t>
+    <t>Multifunktionslenkrad, für Style und FR, Leder</t>
+  </si>
+  <si>
+    <t>Komfortable Türverkleidungen im Innenbereich -</t>
   </si>
   <si>
     <t>Anthrazitfarbene Decke -</t>
   </si>
   <si>
-    <t>Elektrische Fensterheber v orn und h inten, Innenspiegel mit automatischer Blende - -</t>
-  </si>
-  <si>
-    <t>Ambientebeleuchtung im Innenraum, i n den Türen, d er Mittelkonsole und im Fußraum - -</t>
+    <t>Elektrische Fensterheber vorn und hinten, Innenspiegel mit automatischer Blende</t>
+  </si>
+  <si>
+    <t>Ambientebeleuchtung im Innenraum, inden Türen, der Mittelkonsole und im Fußraum</t>
   </si>
   <si>
     <t>Voll-LED-Scheinwerfer mit Tagfahrlicht</t>
   </si>
   <si>
-    <t>Nebelscheinwerfer mit Kurvenlicht (auch f ür Fahrzeuge d er Serien Reference und Style, h ergestellt bis Ende August 2026) - -</t>
+    <t>Nebelscheinwerfer mit Kurvenlicht (auch für Fahrzeuge der Serien Reference und Style, hergestellt bis Ende August 2026)</t>
   </si>
   <si>
     <t>LED-Rückleuchten</t>
   </si>
   <si>
-    <t>Dunkel g etönte Scheiben a b d er B-Säule - -</t>
-  </si>
-  <si>
-    <t>Elektrische Fensterheber v orne -</t>
-  </si>
-  <si>
-    <t>Elektrische Fensterheber v orne und h inten - -</t>
-  </si>
-  <si>
-    <t>Elektrisch verstellbare Außenspiegel, l ackiert, f ür F Rin g länzendem Schwarz</t>
-  </si>
-  <si>
-    <t>Beheizbare Außenspiegel - -</t>
-  </si>
-  <si>
-    <t>Regensensor - -</t>
+    <t>Dunkel getönte Scheiben abder B-Säule</t>
+  </si>
+  <si>
+    <t>Elektrische Fensterheber vorne</t>
+  </si>
+  <si>
+    <t>Elektrische Fensterheber vorne und hinten</t>
+  </si>
+  <si>
+    <t>Elektrisch verstellbare Außenspiegel, lackiert, für FRin glänzendem Schwarz</t>
+  </si>
+  <si>
+    <t>Beheizbare Außenspiegel</t>
+  </si>
+  <si>
+    <t>Regensensor</t>
   </si>
   <si>
     <t>Heckscheibenwischer</t>
@@ -163,19 +163,19 @@
     <t>Einparkhilfe hinten</t>
   </si>
   <si>
-    <t>Einparkhilfe vorn + Rückfahrkamera - -</t>
+    <t>Einparkhilfe vorn + Rückfahrkamera</t>
   </si>
   <si>
     <t>Zentralverriegelung mit Fernbedienung, 15-Zoll-</t>
   </si>
   <si>
-    <t>Stahlfelgen mit 185/65 R 15-Reifen ( Produktion bis M ärz 2026 – 1 5-Zoll-Leichtmetallfelgen), 1 6-Zoll-Leichtmetallfelgen - -</t>
+    <t>Stahlfelgen mit 185/65 R 15-Reifen ( Produktion bis März 2026 – 15-Zoll-Leichtmetallfelgen), 16-Zoll-Leichtmetallfelgen</t>
   </si>
   <si>
     <t>mit 195/55 R 16-Reifen -</t>
   </si>
   <si>
-    <t>Nun m uss der Defekt behoben werden.</t>
+    <t>Nun muss der Defekt behoben werden.</t>
   </si>
   <si>
     <t>_Sicherheit</t>
@@ -197,8 +197,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -214,7 +222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -222,12 +230,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,37 +563,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1346,7 +1372,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1626,7 +1652,7 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C32">
         <v>1</v>

</xml_diff>